<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-06-07 11:04:19
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A1_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A1_session_analysis.xlsx
@@ -806,7 +806,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7">
@@ -916,49 +916,53 @@
         </is>
       </c>
       <c r="L8" s="4" t="n">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>A1-A1</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>07/06/2026</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr"/>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>0/34</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>24/34</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -968,7 +972,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>20.4%</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1025,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>62.9%</t>
+          <t>64.7%</t>
         </is>
       </c>
     </row>
@@ -1306,22 +1310,22 @@
         <v>27</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P15" s="4" t="n">
         <v>2</v>
       </c>
       <c r="Q15" s="4" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>22.2%</t>
         </is>
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>54.7%</t>
+          <t>57.4%</t>
         </is>
       </c>
     </row>
@@ -1384,22 +1388,22 @@
         <v>27</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P16" s="4" t="n">
         <v>2</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>22.2%</t>
         </is>
       </c>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>52.7%</t>
+          <t>59.6%</t>
         </is>
       </c>
     </row>
@@ -1462,22 +1466,22 @@
         <v>27</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P17" s="4" t="n">
         <v>2</v>
       </c>
       <c r="Q17" s="4" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>22.2%</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>68.8%</t>
+          <t>72.5%</t>
         </is>
       </c>
     </row>
@@ -1540,22 +1544,22 @@
         <v>27</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P18" s="4" t="n">
         <v>2</v>
       </c>
       <c r="Q18" s="4" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>22.2%</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>64.2%</t>
         </is>
       </c>
     </row>
@@ -1618,22 +1622,22 @@
         <v>27</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P19" s="4" t="n">
         <v>2</v>
       </c>
       <c r="Q19" s="4" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>22.2%</t>
         </is>
       </c>
       <c r="S19" s="4" t="inlineStr">
         <is>
-          <t>66.5%</t>
+          <t>70.1%</t>
         </is>
       </c>
     </row>
@@ -1696,22 +1700,22 @@
         <v>27</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="R20" s="4" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>22.2%</t>
         </is>
       </c>
       <c r="S20" s="4" t="inlineStr">
         <is>
-          <t>50.9%</t>
+          <t>53.5%</t>
         </is>
       </c>
     </row>
@@ -2656,45 +2660,49 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B36" s="6" t="inlineStr">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>A1-A2</t>
         </is>
       </c>
-      <c r="C36" s="6" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D36" s="6" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E36" s="6" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>07/06/2026</t>
         </is>
       </c>
-      <c r="F36" s="6" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G36" s="6" t="inlineStr"/>
-      <c r="H36" s="6" t="inlineStr">
-        <is>
-          <t>0/33</t>
-        </is>
-      </c>
-      <c r="I36" s="6" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>31/33</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -3837,45 +3845,49 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B63" s="6" t="inlineStr">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
         <is>
           <t>A1-B1</t>
         </is>
       </c>
-      <c r="C63" s="6" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D63" s="6" t="inlineStr">
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E63" s="6" t="inlineStr">
+      <c r="E63" s="2" t="inlineStr">
         <is>
           <t>07/06/2026</t>
         </is>
       </c>
-      <c r="F63" s="6" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G63" s="6" t="inlineStr"/>
-      <c r="H63" s="6" t="inlineStr">
-        <is>
-          <t>0/34</t>
-        </is>
-      </c>
-      <c r="I63" s="6" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>31/34</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -5018,45 +5030,49 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B90" s="6" t="inlineStr">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
         <is>
           <t>A1-B2</t>
         </is>
       </c>
-      <c r="C90" s="6" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D90" s="6" t="inlineStr">
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E90" s="6" t="inlineStr">
+      <c r="E90" s="2" t="inlineStr">
         <is>
           <t>07/06/2026</t>
         </is>
       </c>
-      <c r="F90" s="6" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G90" s="6" t="inlineStr"/>
-      <c r="H90" s="6" t="inlineStr">
-        <is>
-          <t>0/34</t>
-        </is>
-      </c>
-      <c r="I90" s="6" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>29/34</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -6199,45 +6215,49 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B117" s="6" t="inlineStr">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
         <is>
           <t>A1-C1</t>
         </is>
       </c>
-      <c r="C117" s="6" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D117" s="6" t="inlineStr">
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E117" s="6" t="inlineStr">
+      <c r="E117" s="2" t="inlineStr">
         <is>
           <t>07/06/2026</t>
         </is>
       </c>
-      <c r="F117" s="6" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G117" s="6" t="inlineStr"/>
-      <c r="H117" s="6" t="inlineStr">
-        <is>
-          <t>0/34</t>
-        </is>
-      </c>
-      <c r="I117" s="6" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G117" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H117" s="2" t="inlineStr">
+        <is>
+          <t>30/34</t>
+        </is>
+      </c>
+      <c r="I117" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -7380,45 +7400,49 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B144" s="6" t="inlineStr">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
         <is>
           <t>A1-C2</t>
         </is>
       </c>
-      <c r="C144" s="6" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D144" s="6" t="inlineStr">
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E144" s="6" t="inlineStr">
+      <c r="E144" s="2" t="inlineStr">
         <is>
           <t>07/06/2026</t>
         </is>
       </c>
-      <c r="F144" s="6" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G144" s="6" t="inlineStr"/>
-      <c r="H144" s="6" t="inlineStr">
-        <is>
-          <t>0/33</t>
-        </is>
-      </c>
-      <c r="I144" s="6" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H144" s="2" t="inlineStr">
+        <is>
+          <t>22/33</t>
+        </is>
+      </c>
+      <c r="I144" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-06-13 13:47:26
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A1_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A1_session_analysis.xlsx
@@ -806,7 +806,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>90</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7">
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8">
@@ -972,7 +972,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>27.8%</t>
+          <t>29.6%</t>
         </is>
       </c>
     </row>
@@ -1029,50 +1029,54 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>66.1%</t>
+          <t>66.6%</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>A1-A1</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>13/06/2026</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr"/>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>0/34</t>
-        </is>
-      </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>25/34</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -1314,22 +1318,22 @@
         <v>27</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q15" s="4" t="n">
         <v>17</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>25.9%</t>
+          <t>29.6%</t>
         </is>
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>52.1%</t>
+          <t>54.8%</t>
         </is>
       </c>
     </row>
@@ -1392,22 +1396,22 @@
         <v>27</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q16" s="4" t="n">
         <v>17</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>25.9%</t>
+          <t>29.6%</t>
         </is>
       </c>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>56.7%</t>
+          <t>58.0%</t>
         </is>
       </c>
     </row>
@@ -1470,22 +1474,22 @@
         <v>27</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q17" s="4" t="n">
         <v>17</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>25.9%</t>
+          <t>29.6%</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>71.4%</t>
+          <t>72.4%</t>
         </is>
       </c>
     </row>
@@ -1548,22 +1552,22 @@
         <v>27</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>17</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>25.9%</t>
+          <t>29.6%</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>66.8%</t>
+          <t>68.4%</t>
         </is>
       </c>
     </row>
@@ -1626,22 +1630,22 @@
         <v>27</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q19" s="4" t="n">
         <v>17</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>25.9%</t>
+          <t>29.6%</t>
         </is>
       </c>
       <c r="S19" s="4" t="inlineStr">
         <is>
-          <t>71.4%</t>
+          <t>70.2%</t>
         </is>
       </c>
     </row>
@@ -1704,22 +1708,22 @@
         <v>27</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q20" s="4" t="n">
         <v>17</v>
       </c>
       <c r="R20" s="4" t="inlineStr">
         <is>
-          <t>25.9%</t>
+          <t>29.6%</t>
         </is>
       </c>
       <c r="S20" s="4" t="inlineStr">
         <is>
-          <t>56.3%</t>
+          <t>59.5%</t>
         </is>
       </c>
     </row>
@@ -2758,45 +2762,49 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B38" s="5" t="inlineStr">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>A1-A2</t>
         </is>
       </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E38" s="5" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>13/06/2026</t>
         </is>
       </c>
-      <c r="F38" s="5" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G38" s="5" t="inlineStr"/>
-      <c r="H38" s="5" t="inlineStr">
-        <is>
-          <t>0/33</t>
-        </is>
-      </c>
-      <c r="I38" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>22/33</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -3947,45 +3955,49 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B65" s="5" t="inlineStr">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
         <is>
           <t>A1-B1</t>
         </is>
       </c>
-      <c r="C65" s="5" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D65" s="5" t="inlineStr">
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E65" s="5" t="inlineStr">
+      <c r="E65" s="2" t="inlineStr">
         <is>
           <t>13/06/2026</t>
         </is>
       </c>
-      <c r="F65" s="5" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G65" s="5" t="inlineStr"/>
-      <c r="H65" s="5" t="inlineStr">
-        <is>
-          <t>0/34</t>
-        </is>
-      </c>
-      <c r="I65" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>27/34</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -5136,45 +5148,49 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B92" s="5" t="inlineStr">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
         <is>
           <t>A1-B2</t>
         </is>
       </c>
-      <c r="C92" s="5" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D92" s="5" t="inlineStr">
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E92" s="5" t="inlineStr">
+      <c r="E92" s="2" t="inlineStr">
         <is>
           <t>13/06/2026</t>
         </is>
       </c>
-      <c r="F92" s="5" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G92" s="5" t="inlineStr"/>
-      <c r="H92" s="5" t="inlineStr">
-        <is>
-          <t>0/34</t>
-        </is>
-      </c>
-      <c r="I92" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>27/34</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -6325,45 +6341,49 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B119" s="5" t="inlineStr">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
         <is>
           <t>A1-C1</t>
         </is>
       </c>
-      <c r="C119" s="5" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D119" s="5" t="inlineStr">
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E119" s="5" t="inlineStr">
+      <c r="E119" s="2" t="inlineStr">
         <is>
           <t>13/06/2026</t>
         </is>
       </c>
-      <c r="F119" s="5" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G119" s="5" t="inlineStr"/>
-      <c r="H119" s="5" t="inlineStr">
-        <is>
-          <t>0/34</t>
-        </is>
-      </c>
-      <c r="I119" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F119" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G119" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H119" s="2" t="inlineStr">
+        <is>
+          <t>21/34</t>
+        </is>
+      </c>
+      <c r="I119" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -7514,45 +7534,49 @@
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B146" s="5" t="inlineStr">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
         <is>
           <t>A1-C2</t>
         </is>
       </c>
-      <c r="C146" s="5" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D146" s="5" t="inlineStr">
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E146" s="5" t="inlineStr">
+      <c r="E146" s="2" t="inlineStr">
         <is>
           <t>13/06/2026</t>
         </is>
       </c>
-      <c r="F146" s="5" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G146" s="5" t="inlineStr"/>
-      <c r="H146" s="5" t="inlineStr">
-        <is>
-          <t>0/33</t>
-        </is>
-      </c>
-      <c r="I146" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F146" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G146" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H146" s="2" t="inlineStr">
+        <is>
+          <t>27/33</t>
+        </is>
+      </c>
+      <c r="I146" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-06-27 11:24:14
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A1_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A1_session_analysis.xlsx
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>132</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7">
@@ -869,7 +869,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>54</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8">
@@ -980,7 +980,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>40.7%</t>
+          <t>44.4%</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>69.9%</t>
+          <t>70.7%</t>
         </is>
       </c>
     </row>
@@ -1188,45 +1188,49 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>A1-A1</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>20/06/2026</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr"/>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>0/34</t>
-        </is>
-      </c>
-      <c r="I14" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>28/34</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
       <c r="K14" s="1" t="inlineStr">
@@ -1334,22 +1338,22 @@
         <v>27</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q15" s="4" t="n">
         <v>11</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>44.4%</t>
+          <t>51.9%</t>
         </is>
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>64.2%</t>
+          <t>66.2%</t>
         </is>
       </c>
     </row>
@@ -1412,65 +1416,69 @@
         <v>27</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q16" s="4" t="n">
         <v>11</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>44.4%</t>
+          <t>51.9%</t>
         </is>
       </c>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>64.4%</t>
+          <t>67.3%</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>A1-A1</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>27/06/2026</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="inlineStr"/>
-      <c r="H17" s="5" t="inlineStr">
-        <is>
-          <t>0/34</t>
-        </is>
-      </c>
-      <c r="I17" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>25/34</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr">
@@ -1490,22 +1498,22 @@
         <v>27</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q17" s="4" t="n">
         <v>11</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>44.4%</t>
+          <t>51.9%</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>75.7%</t>
+          <t>76.7%</t>
         </is>
       </c>
     </row>
@@ -1568,22 +1576,22 @@
         <v>27</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>11</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>44.4%</t>
+          <t>51.9%</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>73.5%</t>
+          <t>74.6%</t>
         </is>
       </c>
     </row>
@@ -1646,22 +1654,22 @@
         <v>27</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q19" s="4" t="n">
         <v>11</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>44.4%</t>
+          <t>51.9%</t>
         </is>
       </c>
       <c r="S19" s="4" t="inlineStr">
         <is>
-          <t>76.5%</t>
+          <t>76.9%</t>
         </is>
       </c>
     </row>
@@ -1724,22 +1732,22 @@
         <v>27</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q20" s="4" t="n">
         <v>11</v>
       </c>
       <c r="R20" s="4" t="inlineStr">
         <is>
-          <t>44.4%</t>
+          <t>51.9%</t>
         </is>
       </c>
       <c r="S20" s="4" t="inlineStr">
         <is>
-          <t>65.7%</t>
+          <t>66.5%</t>
         </is>
       </c>
     </row>
@@ -2927,45 +2935,49 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="inlineStr">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>A1-A2</t>
         </is>
       </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
-      <c r="E41" s="5" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>20/06/2026</t>
         </is>
       </c>
-      <c r="F41" s="5" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G41" s="5" t="inlineStr"/>
-      <c r="H41" s="5" t="inlineStr">
-        <is>
-          <t>0/33</t>
-        </is>
-      </c>
-      <c r="I41" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>30/33</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -3056,45 +3068,49 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B44" s="5" t="inlineStr">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>A1-A2</t>
         </is>
       </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="E44" s="5" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>27/06/2026</t>
         </is>
       </c>
-      <c r="F44" s="5" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G44" s="5" t="inlineStr"/>
-      <c r="H44" s="5" t="inlineStr">
-        <is>
-          <t>0/33</t>
-        </is>
-      </c>
-      <c r="I44" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>26/33</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -4136,45 +4152,49 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B68" s="5" t="inlineStr">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
         <is>
           <t>A1-B1</t>
         </is>
       </c>
-      <c r="C68" s="5" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D68" s="5" t="inlineStr">
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
-      <c r="E68" s="5" t="inlineStr">
+      <c r="E68" s="2" t="inlineStr">
         <is>
           <t>20/06/2026</t>
         </is>
       </c>
-      <c r="F68" s="5" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G68" s="5" t="inlineStr"/>
-      <c r="H68" s="5" t="inlineStr">
-        <is>
-          <t>0/34</t>
-        </is>
-      </c>
-      <c r="I68" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>26/34</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -4265,45 +4285,49 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B71" s="5" t="inlineStr">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
         <is>
           <t>A1-B1</t>
         </is>
       </c>
-      <c r="C71" s="5" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D71" s="5" t="inlineStr">
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="E71" s="5" t="inlineStr">
+      <c r="E71" s="2" t="inlineStr">
         <is>
           <t>27/06/2026</t>
         </is>
       </c>
-      <c r="F71" s="5" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G71" s="5" t="inlineStr"/>
-      <c r="H71" s="5" t="inlineStr">
-        <is>
-          <t>0/34</t>
-        </is>
-      </c>
-      <c r="I71" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>30/34</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -5345,45 +5369,49 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B95" s="5" t="inlineStr">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
         <is>
           <t>A1-B2</t>
         </is>
       </c>
-      <c r="C95" s="5" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D95" s="5" t="inlineStr">
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
-      <c r="E95" s="5" t="inlineStr">
+      <c r="E95" s="2" t="inlineStr">
         <is>
           <t>20/06/2026</t>
         </is>
       </c>
-      <c r="F95" s="5" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G95" s="5" t="inlineStr"/>
-      <c r="H95" s="5" t="inlineStr">
-        <is>
-          <t>0/34</t>
-        </is>
-      </c>
-      <c r="I95" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>27/34</t>
+        </is>
+      </c>
+      <c r="I95" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -5474,45 +5502,49 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B98" s="5" t="inlineStr">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
         <is>
           <t>A1-B2</t>
         </is>
       </c>
-      <c r="C98" s="5" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D98" s="5" t="inlineStr">
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="E98" s="5" t="inlineStr">
+      <c r="E98" s="2" t="inlineStr">
         <is>
           <t>27/06/2026</t>
         </is>
       </c>
-      <c r="F98" s="5" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G98" s="5" t="inlineStr"/>
-      <c r="H98" s="5" t="inlineStr">
-        <is>
-          <t>0/34</t>
-        </is>
-      </c>
-      <c r="I98" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>28/34</t>
+        </is>
+      </c>
+      <c r="I98" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -6554,45 +6586,49 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B122" s="5" t="inlineStr">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
         <is>
           <t>A1-C1</t>
         </is>
       </c>
-      <c r="C122" s="5" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D122" s="5" t="inlineStr">
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
-      <c r="E122" s="5" t="inlineStr">
+      <c r="E122" s="2" t="inlineStr">
         <is>
           <t>20/06/2026</t>
         </is>
       </c>
-      <c r="F122" s="5" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G122" s="5" t="inlineStr"/>
-      <c r="H122" s="5" t="inlineStr">
-        <is>
-          <t>0/34</t>
-        </is>
-      </c>
-      <c r="I122" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G122" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H122" s="2" t="inlineStr">
+        <is>
+          <t>25/34</t>
+        </is>
+      </c>
+      <c r="I122" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -6683,45 +6719,49 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B125" s="5" t="inlineStr">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
         <is>
           <t>A1-C1</t>
         </is>
       </c>
-      <c r="C125" s="5" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D125" s="5" t="inlineStr">
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="E125" s="5" t="inlineStr">
+      <c r="E125" s="2" t="inlineStr">
         <is>
           <t>27/06/2026</t>
         </is>
       </c>
-      <c r="F125" s="5" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G125" s="5" t="inlineStr"/>
-      <c r="H125" s="5" t="inlineStr">
-        <is>
-          <t>0/34</t>
-        </is>
-      </c>
-      <c r="I125" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G125" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H125" s="2" t="inlineStr">
+        <is>
+          <t>29/34</t>
+        </is>
+      </c>
+      <c r="I125" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -7763,45 +7803,49 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B149" s="5" t="inlineStr">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
         <is>
           <t>A1-C2</t>
         </is>
       </c>
-      <c r="C149" s="5" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D149" s="5" t="inlineStr">
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
-      <c r="E149" s="5" t="inlineStr">
+      <c r="E149" s="2" t="inlineStr">
         <is>
           <t>20/06/2026</t>
         </is>
       </c>
-      <c r="F149" s="5" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G149" s="5" t="inlineStr"/>
-      <c r="H149" s="5" t="inlineStr">
-        <is>
-          <t>0/33</t>
-        </is>
-      </c>
-      <c r="I149" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F149" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G149" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H149" s="2" t="inlineStr">
+        <is>
+          <t>22/33</t>
+        </is>
+      </c>
+      <c r="I149" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -7892,45 +7936,49 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B152" s="5" t="inlineStr">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
         <is>
           <t>A1-C2</t>
         </is>
       </c>
-      <c r="C152" s="5" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D152" s="5" t="inlineStr">
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="E152" s="5" t="inlineStr">
+      <c r="E152" s="2" t="inlineStr">
         <is>
           <t>27/06/2026</t>
         </is>
       </c>
-      <c r="F152" s="5" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G152" s="5" t="inlineStr"/>
-      <c r="H152" s="5" t="inlineStr">
-        <is>
-          <t>0/33</t>
-        </is>
-      </c>
-      <c r="I152" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F152" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G152" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H152" s="2" t="inlineStr">
+        <is>
+          <t>25/33</t>
+        </is>
+      </c>
+      <c r="I152" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-06-27 13:21:13
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A1_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Surgery_1_A1_session_analysis.xlsx
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
     </row>
     <row r="7">
@@ -869,7 +869,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>42</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8">
@@ -980,7 +980,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>44.4%</t>
+          <t>46.3%</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>70.7%</t>
+          <t>71.8%</t>
         </is>
       </c>
     </row>
@@ -1280,45 +1280,49 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>A1-A1</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>21/06/2026</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr"/>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>0/34</t>
-        </is>
-      </c>
-      <c r="I15" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>34/34</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr">
@@ -1338,22 +1342,22 @@
         <v>27</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q15" s="4" t="n">
         <v>11</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>51.9%</t>
+          <t>55.6%</t>
         </is>
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>66.2%</t>
+          <t>68.4%</t>
         </is>
       </c>
     </row>
@@ -1416,22 +1420,22 @@
         <v>27</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q16" s="4" t="n">
         <v>11</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>51.9%</t>
+          <t>55.6%</t>
         </is>
       </c>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>67.3%</t>
+          <t>69.5%</t>
         </is>
       </c>
     </row>
@@ -1498,22 +1502,22 @@
         <v>27</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q17" s="4" t="n">
         <v>11</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>51.9%</t>
+          <t>55.6%</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>76.7%</t>
+          <t>78.2%</t>
         </is>
       </c>
     </row>
@@ -1576,22 +1580,22 @@
         <v>27</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>11</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>51.9%</t>
+          <t>55.6%</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>74.6%</t>
+          <t>76.3%</t>
         </is>
       </c>
     </row>
@@ -1654,22 +1658,22 @@
         <v>27</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q19" s="4" t="n">
         <v>11</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>51.9%</t>
+          <t>55.6%</t>
         </is>
       </c>
       <c r="S19" s="4" t="inlineStr">
         <is>
-          <t>76.9%</t>
+          <t>78.4%</t>
         </is>
       </c>
     </row>
@@ -1732,22 +1736,22 @@
         <v>27</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q20" s="4" t="n">
         <v>11</v>
       </c>
       <c r="R20" s="4" t="inlineStr">
         <is>
-          <t>51.9%</t>
+          <t>55.6%</t>
         </is>
       </c>
       <c r="S20" s="4" t="inlineStr">
         <is>
-          <t>66.5%</t>
+          <t>68.7%</t>
         </is>
       </c>
     </row>
@@ -2982,45 +2986,49 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>A1-A2</t>
         </is>
       </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="E42" s="5" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>21/06/2026</t>
         </is>
       </c>
-      <c r="F42" s="5" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G42" s="5" t="inlineStr"/>
-      <c r="H42" s="5" t="inlineStr">
-        <is>
-          <t>0/33</t>
-        </is>
-      </c>
-      <c r="I42" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>33/33</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -4199,45 +4207,49 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B69" s="5" t="inlineStr">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
         <is>
           <t>A1-B1</t>
         </is>
       </c>
-      <c r="C69" s="5" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D69" s="5" t="inlineStr">
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="E69" s="5" t="inlineStr">
+      <c r="E69" s="2" t="inlineStr">
         <is>
           <t>21/06/2026</t>
         </is>
       </c>
-      <c r="F69" s="5" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G69" s="5" t="inlineStr"/>
-      <c r="H69" s="5" t="inlineStr">
-        <is>
-          <t>0/34</t>
-        </is>
-      </c>
-      <c r="I69" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>34/34</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -5416,45 +5428,49 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B96" s="5" t="inlineStr">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
         <is>
           <t>A1-B2</t>
         </is>
       </c>
-      <c r="C96" s="5" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D96" s="5" t="inlineStr">
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="E96" s="5" t="inlineStr">
+      <c r="E96" s="2" t="inlineStr">
         <is>
           <t>21/06/2026</t>
         </is>
       </c>
-      <c r="F96" s="5" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G96" s="5" t="inlineStr"/>
-      <c r="H96" s="5" t="inlineStr">
-        <is>
-          <t>0/34</t>
-        </is>
-      </c>
-      <c r="I96" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>34/34</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -6633,45 +6649,49 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B123" s="5" t="inlineStr">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
         <is>
           <t>A1-C1</t>
         </is>
       </c>
-      <c r="C123" s="5" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D123" s="5" t="inlineStr">
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="E123" s="5" t="inlineStr">
+      <c r="E123" s="2" t="inlineStr">
         <is>
           <t>21/06/2026</t>
         </is>
       </c>
-      <c r="F123" s="5" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G123" s="5" t="inlineStr"/>
-      <c r="H123" s="5" t="inlineStr">
-        <is>
-          <t>0/34</t>
-        </is>
-      </c>
-      <c r="I123" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F123" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G123" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H123" s="2" t="inlineStr">
+        <is>
+          <t>34/34</t>
+        </is>
+      </c>
+      <c r="I123" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -7850,45 +7870,49 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B150" s="5" t="inlineStr">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
         <is>
           <t>A1-C2</t>
         </is>
       </c>
-      <c r="C150" s="5" t="inlineStr">
-        <is>
-          <t>GENERAL SURGERY</t>
-        </is>
-      </c>
-      <c r="D150" s="5" t="inlineStr">
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL SURGERY</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="E150" s="5" t="inlineStr">
+      <c r="E150" s="2" t="inlineStr">
         <is>
           <t>21/06/2026</t>
         </is>
       </c>
-      <c r="F150" s="5" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="G150" s="5" t="inlineStr"/>
-      <c r="H150" s="5" t="inlineStr">
-        <is>
-          <t>0/33</t>
-        </is>
-      </c>
-      <c r="I150" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F150" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="G150" s="2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H150" s="2" t="inlineStr">
+        <is>
+          <t>33/33</t>
+        </is>
+      </c>
+      <c r="I150" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>